<commit_message>
10-Oct-2025 Stock market report
Here i was attached stock market profit and loss report
</commit_message>
<xml_diff>
--- a/ShareMarket-2025.xlsx
+++ b/ShareMarket-2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8100000_{0FA1F1E3-9754-430C-80B6-13A2687C9C41}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8100000_{6C03CD62-EEDF-4F5A-983D-4D769AEB63BC}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8952" activeTab="4" xr2:uid="{ED50D364-8611-4D83-A6B8-5F797ED4AD3A}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="123">
   <si>
     <t>S.NO</t>
   </si>
@@ -488,6 +488,38 @@
   </si>
   <si>
     <t>0/507</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Adobe Fan Heiti Std B"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>622</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF9C0006"/>
+        <rFont val="Adobe Fan Heiti Std B"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Adobe Fan Heiti Std B"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>-400</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1167,6 +1199,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="60" fillId="2" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="64" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1176,9 +1211,6 @@
     </xf>
     <xf numFmtId="0" fontId="59" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="64" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -3334,14 +3366,14 @@
         <v>53</v>
       </c>
       <c r="C9" s="24">
-        <v>250</v>
-      </c>
-      <c r="D9" s="33" t="s">
-        <v>102</v>
+        <v>500</v>
+      </c>
+      <c r="D9" s="33">
+        <v>45726</v>
       </c>
       <c r="E9" s="24"/>
       <c r="F9" s="25">
-        <v>91.39</v>
+        <v>96.84</v>
       </c>
       <c r="G9" s="24">
         <v>0</v>
@@ -3354,7 +3386,7 @@
       </c>
       <c r="J9" s="27">
         <f t="shared" si="2"/>
-        <v>22847.5</v>
+        <v>48420</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="25.8" x14ac:dyDescent="0.5">
@@ -3827,13 +3859,13 @@
       <c r="E17" s="6">
         <v>229.02</v>
       </c>
-      <c r="L17" s="108" t="s">
+      <c r="L17" s="109" t="s">
         <v>10</v>
       </c>
-      <c r="M17" s="108"/>
-      <c r="N17" s="108"/>
-      <c r="O17" s="108"/>
-      <c r="P17" s="108"/>
+      <c r="M17" s="109"/>
+      <c r="N17" s="109"/>
+      <c r="O17" s="109"/>
+      <c r="P17" s="109"/>
     </row>
     <row r="18" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
@@ -3851,11 +3883,11 @@
       <c r="E18" s="6">
         <v>101.04</v>
       </c>
-      <c r="L18" s="108"/>
-      <c r="M18" s="108"/>
-      <c r="N18" s="108"/>
-      <c r="O18" s="108"/>
-      <c r="P18" s="108"/>
+      <c r="L18" s="109"/>
+      <c r="M18" s="109"/>
+      <c r="N18" s="109"/>
+      <c r="O18" s="109"/>
+      <c r="P18" s="109"/>
     </row>
     <row r="19" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
@@ -4816,19 +4848,19 @@
   </cols>
   <sheetData>
     <row r="2" spans="5:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G2" s="109"/>
-      <c r="H2" s="109"/>
-      <c r="I2" s="109"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
     </row>
     <row r="3" spans="5:10" x14ac:dyDescent="0.3">
-      <c r="G3" s="109"/>
-      <c r="H3" s="109"/>
-      <c r="I3" s="109"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
     </row>
     <row r="4" spans="5:10" x14ac:dyDescent="0.3">
-      <c r="G4" s="109"/>
-      <c r="H4" s="109"/>
-      <c r="I4" s="109"/>
+      <c r="G4" s="110"/>
+      <c r="H4" s="110"/>
+      <c r="I4" s="110"/>
     </row>
     <row r="5" spans="5:10" ht="36.6" x14ac:dyDescent="0.7">
       <c r="E5" s="102"/>
@@ -4837,10 +4869,10 @@
       </c>
       <c r="G5" s="107"/>
       <c r="H5" s="106"/>
-      <c r="I5" s="110" t="s">
+      <c r="I5" s="111" t="s">
         <v>119</v>
       </c>
-      <c r="J5" s="111"/>
+      <c r="J5" s="112"/>
     </row>
     <row r="6" spans="5:10" ht="21.6" x14ac:dyDescent="0.45">
       <c r="F6" s="10" t="s">
@@ -4872,7 +4904,7 @@
       <c r="I8" s="103" t="s">
         <v>117</v>
       </c>
-      <c r="J8" s="112">
+      <c r="J8" s="108">
         <v>80</v>
       </c>
     </row>
@@ -4889,7 +4921,7 @@
       <c r="I9" s="103" t="s">
         <v>109</v>
       </c>
-      <c r="J9" s="112">
+      <c r="J9" s="108">
         <v>80</v>
       </c>
     </row>
@@ -4906,7 +4938,7 @@
       <c r="I10" s="103" t="s">
         <v>117</v>
       </c>
-      <c r="J10" s="112">
+      <c r="J10" s="108">
         <v>120</v>
       </c>
     </row>
@@ -4923,7 +4955,7 @@
       <c r="I11" s="103" t="s">
         <v>116</v>
       </c>
-      <c r="J11" s="112">
+      <c r="J11" s="108">
         <v>100</v>
       </c>
     </row>
@@ -4941,7 +4973,7 @@
       <c r="I12" s="103" t="s">
         <v>115</v>
       </c>
-      <c r="J12" s="112">
+      <c r="J12" s="108">
         <v>120</v>
       </c>
     </row>
@@ -4958,7 +4990,7 @@
       <c r="I13" s="103" t="s">
         <v>114</v>
       </c>
-      <c r="J13" s="112">
+      <c r="J13" s="108">
         <v>100</v>
       </c>
     </row>
@@ -4975,7 +5007,7 @@
       <c r="I14" s="105">
         <v>45667</v>
       </c>
-      <c r="J14" s="112">
+      <c r="J14" s="108">
         <v>70</v>
       </c>
     </row>
@@ -4992,7 +5024,7 @@
       <c r="I15" s="105">
         <v>45726</v>
       </c>
-      <c r="J15" s="112">
+      <c r="J15" s="108">
         <v>60</v>
       </c>
     </row>
@@ -5009,7 +5041,7 @@
       <c r="I16" s="105">
         <v>45818</v>
       </c>
-      <c r="J16" s="112">
+      <c r="J16" s="108">
         <v>90</v>
       </c>
     </row>
@@ -5026,7 +5058,7 @@
       <c r="I17" s="105">
         <v>45848</v>
       </c>
-      <c r="J17" s="112">
+      <c r="J17" s="108">
         <v>100</v>
       </c>
     </row>
@@ -5043,7 +5075,7 @@
       <c r="I18" s="105">
         <v>45879</v>
       </c>
-      <c r="J18" s="112" t="s">
+      <c r="J18" s="108" t="s">
         <v>121</v>
       </c>
     </row>
@@ -5064,11 +5096,22 @@
         <v>120</v>
       </c>
     </row>
-    <row r="20" spans="6:10" ht="21.6" x14ac:dyDescent="0.45">
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
+    <row r="20" spans="6:10" ht="18.600000000000001" x14ac:dyDescent="0.4">
+      <c r="F20" s="97">
+        <v>12</v>
+      </c>
+      <c r="G20" s="101">
+        <v>45940</v>
+      </c>
+      <c r="H20" s="97">
+        <v>320</v>
+      </c>
+      <c r="I20" s="105">
+        <v>45940</v>
+      </c>
+      <c r="J20" s="104" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="21" spans="6:10" ht="21.6" x14ac:dyDescent="0.45">
       <c r="F21" s="8"/>

</xml_diff>